<commit_message>
Updated testcases to include additional tabs
</commit_message>
<xml_diff>
--- a/InputFiles/C3DC/TC01_C3DC_phs002790_SexAtBirth-Female.xlsx
+++ b/InputFiles/C3DC/TC01_C3DC_phs002790_SexAtBirth-Female.xlsx
@@ -507,31 +507,82 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>SELECT DISTINCT
-     std.dbgap_accession AS "dbGaP Accession",
-     std.study_name AS "Study Name"
-FROM 
-    df_study std
-LEFT JOIN 
-    df_participant prt 
-        ON 1=1   -- participants not directly linked to studies
-LEFT JOIN 
-    df_diagnoses dgn 
-        ON prt.id = dgn."participant.id"
-LEFT JOIN 
-    df_treatments trt 
-        ON prt.id = trt."participant.id"
-LEFT JOIN 
-    df_treatment_resp trr 
-        ON prt.id = trr."participant.id"
-LEFT JOIN 
-    df_survival srv 
-        ON prt.id = srv."participant.id"
-LEFT JOIN 
-    df_genetic_analyses ga 
-        ON prt.id = ga."participant.id"
-WHERE 
-    std.dbgap_accession = 'phs003164' AND prt.sex_at_birth = 'phs002790'</t>
+          <t>MATCH (s:study)
+WHERE EXISTS {
+  MATCH (p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+  WHERE s.dbgap_accession = 'phs002790' AND p.sex_at_birth = 'Female'
+}
+WITH s
+MATCH (sp:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+WITH s, count(DISTINCT sp) AS num_of_participants
+OPTIONAL MATCH (sm:sample)-[:of_sample]-&gt;(:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+WITH s, num_of_participants, count(DISTINCT sm) AS num_of_samples
+OPTIONAL MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(dp:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+WITH s, num_of_participants, num_of_samples, d.diagnosis AS diagnosis_name, count(DISTINCT dp) AS diagnosis_n
+ORDER BY diagnosis_n DESC, diagnosis_name
+WITH s, num_of_participants, num_of_samples,
+     [item IN collect(CASE WHEN diagnosis_name IS NULL THEN null ELSE diagnosis_name + ' (' + toString(diagnosis_n) + ')' END) WHERE item IS NOT NULL] AS diagnosis_all
+WITH s, num_of_participants, num_of_samples,
+     diagnosis_all[0..5] AS diagnosis_items,
+     size(diagnosis_all) &gt; 5 AS diagnosis_more
+OPTIONAL MATCH (d2:diagnosis)-[:of_diagnosis]-&gt;(dp2:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+UNWIND CASE WHEN d2 IS NULL THEN [null] ELSE coalesce(d2.anatomic_site, [null]) END AS site
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site, count(DISTINCT dp2) AS site_n
+ORDER BY site_n DESC, site
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more,
+     [item IN collect(CASE WHEN site IS NULL THEN null ELSE site + ' (' + toString(site_n) + ')' END) WHERE item IS NOT NULL] AS site_all
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more,
+     site_all[0..5] AS site_items,
+     size(site_all) &gt; 5 AS site_more
+OPTIONAL MATCH (sf)-[:of_sequencing_file|of_clinical_measure_file|of_cytogenomic_file|of_generic_file|of_methylation_array_file|of_pathology_file]-&gt;(:sample)-[:of_sample]-&gt;(:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more,
+     sf.file_type AS file_type, count(DISTINCT sf) AS type_n
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more,
+     [item IN collect(CASE WHEN file_type IS NULL OR type_n = 0 THEN null ELSE {t: file_type, n: type_n} END) WHERE item IS NOT NULL] AS sample_file_types
+OPTIONAL MATCH (pf)-[:of_clinical_measure_file|of_generic_file|of_radiology_file]-&gt;(:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, sample_file_types,
+     pf.file_type AS file_type, count(DISTINCT pf) AS type_n
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, sample_file_types,
+     [item IN collect(CASE WHEN file_type IS NULL OR type_n = 0 THEN null ELSE {t: file_type, n: type_n} END) WHERE item IS NOT NULL] AS participant_file_types
+OPTIONAL MATCH (stf)-[:of_clinical_measure_file|of_generic_file]-&gt;(s)
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, sample_file_types, participant_file_types,
+     stf.file_type AS file_type, count(DISTINCT stf) AS type_n
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more,
+     sample_file_types + participant_file_types + [item IN collect(CASE WHEN file_type IS NULL OR type_n = 0 THEN null ELSE {t: file_type, n: type_n} END) WHERE item IS NOT NULL] AS file_types
+UNWIND CASE WHEN size(file_types) = 0 THEN [{t: null, n: 0}] ELSE file_types END AS ft
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more,
+     ft.t AS file_type, sum(ft.n) AS type_n
+ORDER BY type_n DESC, file_type
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more,
+     sum(CASE WHEN file_type IS NULL THEN 0 ELSE type_n END) AS num_of_files,
+     [item IN collect(CASE WHEN file_type IS NULL THEN null ELSE file_type + ' (' + toString(type_n) + ')' END) WHERE item IS NOT NULL] AS file_type_all
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, num_of_files,
+     file_type_all[0..5] AS file_type_items,
+     size(file_type_all) &gt; 5 AS file_type_more
+OPTIONAL MATCH (pub:publication)-[:of_publication]-&gt;(s)
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, num_of_files, file_type_items, file_type_more,
+     [id IN collect(pub.pubmed_id) WHERE id IS NOT NULL] AS pubmed_ids
+OPTIONAL MATCH (per:study_personnel)-[:of_study_personnel]-&gt;(s)
+WHERE per IS NULL OR per.personnel_type = 'PI'
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, num_of_files, file_type_items, file_type_more, pubmed_ids,
+     [name IN collect(per.personnel_name) WHERE name IS NOT NULL] AS investigators
+OPTIONAL MATCH (fund:study_funding)-[:of_study_funding]-&gt;(s)
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, num_of_files, file_type_items, file_type_more, pubmed_ids, investigators,
+     [id IN collect(fund.grant_id) WHERE id IS NOT NULL] AS grant_ids
+RETURN s.study_name AS `Study Name`,
+       s.study_id AS `Study ID`,
+       s.study_phase AS `Study Phase`,
+       reduce(text = '', item IN diagnosis_items | CASE WHEN text = '' THEN item ELSE text + '\u000a' + item END) + CASE WHEN diagnosis_more THEN '\u000a' + 'Read More' ELSE '' END AS `Diagnosis (Top 5)`,
+       reduce(text = '', item IN site_items | CASE WHEN text = '' THEN item ELSE text + '\u000a' + item END) + CASE WHEN site_more THEN '\u000a' + 'Read More' ELSE '' END AS `Diagnosis Anatomic Site (Top 5)`,
+       toString(num_of_participants) AS `Number of Participants`,
+       toString(num_of_samples) AS `Number of Samples`,
+       toString(num_of_files) AS `Number of Files`,
+       reduce(text = '', item IN file_type_items | CASE WHEN text = '' THEN item ELSE text + '\u000a' + item END) + CASE WHEN file_type_more THEN '\u000a' + 'Read More' ELSE '' END AS `File Type (Top 5)`,
+       reduce(text = '', item IN pubmed_ids | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS `PubMed ID`,
+       reduce(text = '', item IN investigators | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS `Principal Investigator(s)`,
+       reduce(text = '', item IN grant_ids | CASE WHEN text = '' THEN item ELSE text + ', ' + item END) AS `Grant ID`
+ORDER BY s.study_name
+LIMIT 100;</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">

</xml_diff>